<commit_message>
data: canonicalise case risks and refresh case corpus / evaluation outputs
- case_database_v0.1: related_risk now in the Task 1 six-category order,
  RETURN_003 Cost Risk dropped, NEWS_004/007/013 links verified
- raw/case/*.md regenerated so the corpus matches the workbook
- evaluation/* recomputed after the case-corpus refresh (metrics unchanged:
  risk recall 0.461 / precision 0.676, citation completeness 100%)
</commit_message>
<xml_diff>
--- a/data/evaluation/evidence_quality_test.xlsx
+++ b/data/evaluation/evidence_quality_test.xlsx
@@ -8559,17 +8559,17 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>PLUS1_002</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>东方财富网（转界面新闻）</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>2024-07-16</t>
+          <t>2025-07-02</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
@@ -8594,7 +8594,7 @@
       </c>
       <c r="L156" s="2" t="inlineStr">
         <is>
-          <t>https://finance.eastmoney.com/a/202407163131488556.html</t>
+          <t>https://finance.eastmoney.com/a/202507023446498365.html</t>
         </is>
       </c>
     </row>
@@ -8819,17 +8819,17 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>PLUS1_002</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>东方财富网（转界面新闻）</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>2024-07-16</t>
+          <t>2025-07-02</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="L161" s="2" t="inlineStr">
         <is>
-          <t>https://finance.eastmoney.com/a/202407163131488556.html</t>
+          <t>https://finance.eastmoney.com/a/202507023446498365.html</t>
         </is>
       </c>
     </row>

</xml_diff>